<commit_message>
Move Inputs for completed challenges to Done folder (2015)
</commit_message>
<xml_diff>
--- a/Documents/AdventStats.xlsx
+++ b/Documents/AdventStats.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Userfiles\Hobbies\Computer\Sources\Advent\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Hobbies\Computer\Sources\Advent\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09E7A559-0265-4453-95A3-85FFD526C580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80DE8043-40D1-4290-B5B1-F6E64FAC68D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="450" windowWidth="10506" windowHeight="11502" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2820" yWindow="5100" windowWidth="25515" windowHeight="15885" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2024" sheetId="12" r:id="rId1"/>
@@ -29,6 +29,20 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -663,14 +677,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2AA6AC8-5A6F-44C5-8B15-8AB7181E67FD}">
   <dimension ref="A1:K26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="10.26171875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.68359375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.1015625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -705,7 +719,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -743,7 +757,7 @@
       </c>
       <c r="K2" s="2"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <f>A2+1</f>
         <v>2</v>
@@ -784,7 +798,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" ref="A4:A26" si="4">A3+1</f>
         <v>3</v>
@@ -823,7 +837,7 @@
       </c>
       <c r="K4" s="2"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="4"/>
         <v>4</v>
@@ -862,7 +876,7 @@
       </c>
       <c r="K5" s="2"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="4"/>
         <v>5</v>
@@ -901,7 +915,7 @@
       </c>
       <c r="K6" s="2"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7">
         <f t="shared" si="4"/>
         <v>6</v>
@@ -940,7 +954,7 @@
       </c>
       <c r="K7" s="2"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8">
         <f t="shared" si="4"/>
         <v>7</v>
@@ -979,7 +993,7 @@
       </c>
       <c r="K8" s="2"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9">
         <f t="shared" si="4"/>
         <v>8</v>
@@ -1020,7 +1034,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10">
         <f t="shared" si="4"/>
         <v>9</v>
@@ -1059,7 +1073,7 @@
       </c>
       <c r="K10" s="2"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11">
         <f t="shared" si="4"/>
         <v>10</v>
@@ -1098,7 +1112,7 @@
       </c>
       <c r="K11" s="2"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12">
         <f t="shared" si="4"/>
         <v>11</v>
@@ -1137,7 +1151,7 @@
       </c>
       <c r="K12" s="2"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13">
         <f t="shared" si="4"/>
         <v>12</v>
@@ -1176,7 +1190,7 @@
       </c>
       <c r="K13" s="2"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14">
         <f t="shared" si="4"/>
         <v>13</v>
@@ -1215,7 +1229,7 @@
       </c>
       <c r="K14" s="2"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15">
         <f t="shared" si="4"/>
         <v>14</v>
@@ -1254,7 +1268,7 @@
       </c>
       <c r="K15" s="2"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16">
         <f t="shared" si="4"/>
         <v>15</v>
@@ -1293,7 +1307,7 @@
       </c>
       <c r="K16" s="2"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17">
         <f t="shared" si="4"/>
         <v>16</v>
@@ -1332,7 +1346,7 @@
       </c>
       <c r="K17" s="2"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18">
         <f t="shared" si="4"/>
         <v>17</v>
@@ -1371,7 +1385,7 @@
       </c>
       <c r="K18" s="2"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19">
         <f t="shared" si="4"/>
         <v>18</v>
@@ -1410,7 +1424,7 @@
       </c>
       <c r="K19" s="2"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20">
         <f t="shared" si="4"/>
         <v>19</v>
@@ -1451,7 +1465,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21">
         <f t="shared" si="4"/>
         <v>20</v>
@@ -1490,7 +1504,7 @@
       </c>
       <c r="K21" s="2"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22">
         <f t="shared" si="4"/>
         <v>21</v>
@@ -1527,7 +1541,7 @@
       </c>
       <c r="K22" s="2"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23">
         <f t="shared" si="4"/>
         <v>22</v>
@@ -1566,7 +1580,7 @@
       </c>
       <c r="K23" s="2"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24">
         <f t="shared" si="4"/>
         <v>23</v>
@@ -1603,7 +1617,7 @@
       </c>
       <c r="K24" s="2"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25">
         <f t="shared" si="4"/>
         <v>24</v>
@@ -1640,7 +1654,7 @@
       </c>
       <c r="K25" s="2"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26">
         <f t="shared" si="4"/>
         <v>25</v>
@@ -1739,13 +1753,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:J28"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="7" max="8" width="9.15625" style="1"/>
-    <col min="10" max="10" width="11.15625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="9.140625" style="1"/>
+    <col min="10" max="10" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1777,7 +1791,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1814,7 +1828,7 @@
         <v>0.19781078967943705</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
         <f>A2+1</f>
         <v>2</v>
@@ -1852,7 +1866,7 @@
         <v>8.9479628181739213E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" ref="A4:A26" si="5">A3+1</f>
         <v>3</v>
@@ -1890,7 +1904,7 @@
         <v>9.247676135870038E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="5"/>
         <v>4</v>
@@ -1928,7 +1942,7 @@
         <v>0.20767092346451221</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="5"/>
         <v>5</v>
@@ -1966,7 +1980,7 @@
         <v>0.19980887846407783</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7">
         <f t="shared" si="5"/>
         <v>6</v>
@@ -2004,7 +2018,7 @@
         <v>0.20332725219355399</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8">
         <f t="shared" si="5"/>
         <v>7</v>
@@ -2042,7 +2056,7 @@
         <v>8.387629224220311E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9">
         <f t="shared" si="5"/>
         <v>8</v>
@@ -2080,7 +2094,7 @@
         <v>9.70376161932065E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10">
         <f t="shared" si="5"/>
         <v>9</v>
@@ -2118,7 +2132,7 @@
         <v>7.1453392407262617E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11">
         <f t="shared" si="5"/>
         <v>10</v>
@@ -2156,7 +2170,7 @@
         <v>5.7206150638519679E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12">
         <f t="shared" si="5"/>
         <v>11</v>
@@ -2194,7 +2208,7 @@
         <v>4.7302580140734948E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13">
         <f t="shared" si="5"/>
         <v>12</v>
@@ -2232,7 +2246,7 @@
         <v>8.066197550169403E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14">
         <f t="shared" si="5"/>
         <v>13</v>
@@ -2270,7 +2284,7 @@
         <v>4.2741725306228821E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15">
         <f t="shared" si="5"/>
         <v>14</v>
@@ -2308,7 +2322,7 @@
         <v>6.6631917296499005E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16">
         <f t="shared" si="5"/>
         <v>15</v>
@@ -2346,7 +2360,7 @@
         <v>4.8171314394926591E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17">
         <f t="shared" si="5"/>
         <v>16</v>
@@ -2384,7 +2398,7 @@
         <v>6.7109721136304409E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18">
         <f t="shared" si="5"/>
         <v>17</v>
@@ -2422,7 +2436,7 @@
         <v>5.1950308400660235E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19">
         <f t="shared" si="5"/>
         <v>18</v>
@@ -2460,7 +2474,7 @@
         <v>8.066197550169403E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20">
         <f t="shared" si="5"/>
         <v>19</v>
@@ -2498,7 +2512,7 @@
         <v>6.5632872904178616E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21">
         <f t="shared" si="5"/>
         <v>20</v>
@@ -2536,7 +2550,7 @@
         <v>6.1332638345929981E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22">
         <f t="shared" si="5"/>
         <v>21</v>
@@ -2574,7 +2588,7 @@
         <v>6.5111632351663631E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23">
         <f t="shared" si="5"/>
         <v>22</v>
@@ -2612,7 +2626,7 @@
         <v>2.6626704890973851E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24">
         <f t="shared" si="5"/>
         <v>23</v>
@@ -2650,7 +2664,7 @@
         <v>7.1453392407262617E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25">
         <f t="shared" si="5"/>
         <v>24</v>
@@ -2688,7 +2702,7 @@
         <v>6.0029536964642513E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26">
         <f t="shared" si="5"/>
         <v>25</v>
@@ -2726,13 +2740,13 @@
         <v>5.2601859091303972E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="I27" s="1" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="I28" s="1" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -2787,13 +2801,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:J28"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="7" max="8" width="9.15625" style="1"/>
-    <col min="10" max="10" width="11.15625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="9.140625" style="1"/>
+    <col min="10" max="10" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2825,7 +2839,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2862,7 +2876,7 @@
         <v>0.35516871268531564</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
         <f>A2+1</f>
         <v>2</v>
@@ -2900,7 +2914,7 @@
         <v>0.26519420406520428</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" ref="A4:A26" si="4">A3+1</f>
         <v>3</v>
@@ -2938,7 +2952,7 @@
         <v>0.21749849064198029</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="4"/>
         <v>4</v>
@@ -2976,7 +2990,7 @@
         <v>0.19142013819011203</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="4"/>
         <v>5</v>
@@ -3014,7 +3028,7 @@
         <v>0.15774468370564165</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7">
         <f t="shared" si="4"/>
         <v>6</v>
@@ -3052,7 +3066,7 @@
         <v>0.14031998390018113</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8">
         <f t="shared" si="4"/>
         <v>7</v>
@@ -3090,7 +3104,7 @@
         <v>9.4636747836586835E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9">
         <f t="shared" si="4"/>
         <v>8</v>
@@ -3128,7 +3142,7 @@
         <v>8.9672637016166901E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10">
         <f t="shared" si="4"/>
         <v>9</v>
@@ -3166,7 +3180,7 @@
         <v>7.9459314416046159E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11">
         <f t="shared" si="4"/>
         <v>10</v>
@@ -3204,7 +3218,7 @@
         <v>9.3831756892734958E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12">
         <f t="shared" si="4"/>
         <v>11</v>
@@ -3242,7 +3256,7 @@
         <v>7.5132488092842287E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13">
         <f t="shared" si="4"/>
         <v>12</v>
@@ -3280,7 +3294,7 @@
         <v>6.5623532568591936E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14">
         <f t="shared" si="4"/>
         <v>13</v>
@@ -3318,7 +3332,7 @@
         <v>6.4701147112094987E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15">
         <f t="shared" si="4"/>
         <v>14</v>
@@ -3356,7 +3370,7 @@
         <v>6.2084926544576376E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16">
         <f t="shared" si="4"/>
         <v>15</v>
@@ -3394,7 +3408,7 @@
         <v>6.2990541356409746E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17">
         <f t="shared" si="4"/>
         <v>16</v>
@@ -3432,7 +3446,7 @@
         <v>6.4885624203394374E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18">
         <f t="shared" si="4"/>
         <v>17</v>
@@ -3470,7 +3484,7 @@
         <v>5.8965586637150333E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19">
         <f t="shared" si="4"/>
         <v>18</v>
@@ -3508,7 +3522,7 @@
         <v>5.5410209968471187E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20">
         <f t="shared" si="4"/>
         <v>19</v>
@@ -3546,7 +3560,7 @@
         <v>3.9075602066143425E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21">
         <f t="shared" si="4"/>
         <v>20</v>
@@ -3584,7 +3598,7 @@
         <v>4.4274501911853489E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22">
         <f t="shared" si="4"/>
         <v>21</v>
@@ -3622,7 +3636,7 @@
         <v>4.0886831689810159E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23">
         <f t="shared" si="4"/>
         <v>22</v>
@@ -3660,7 +3674,7 @@
         <v>2.9415710739920841E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24">
         <f t="shared" si="4"/>
         <v>23</v>
@@ -3698,7 +3712,7 @@
         <v>3.867310659421748E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25">
         <f t="shared" si="4"/>
         <v>24</v>
@@ -3736,7 +3750,7 @@
         <v>2.9969142013819013E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26">
         <f t="shared" si="4"/>
         <v>25</v>
@@ -3774,13 +3788,13 @@
         <v>2.5742939558596634E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="J27" s="1" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="J28" s="1" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -3858,14 +3872,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76543402-6771-4C6D-98B2-2473D542FE19}">
   <dimension ref="A1:CZ22"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="101" width="1.68359375" customWidth="1"/>
+    <col min="2" max="101" width="1.7109375" customWidth="1"/>
     <col min="102" max="102" width="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:104" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:104" x14ac:dyDescent="0.25">
       <c r="B1" s="12">
         <v>1</v>
       </c>
@@ -4017,7 +4031,7 @@
       <c r="CV1" s="12"/>
       <c r="CW1" s="12"/>
     </row>
-    <row r="2" spans="1:104" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:104" x14ac:dyDescent="0.25">
       <c r="B2" s="12" t="s">
         <v>12</v>
       </c>
@@ -4219,7 +4233,7 @@
       </c>
       <c r="CW2" s="12"/>
     </row>
-    <row r="3" spans="1:104" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:104" x14ac:dyDescent="0.25">
       <c r="B3">
         <v>1</v>
       </c>
@@ -4521,7 +4535,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:104" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:104" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2015</v>
       </c>
@@ -4745,13 +4759,13 @@
         <v>14</v>
       </c>
       <c r="BW4" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="BX4" s="2" t="s">
         <v>14</v>
       </c>
       <c r="BY4" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="BZ4" s="2" t="s">
         <v>14</v>
@@ -4760,10 +4774,10 @@
         <v>14</v>
       </c>
       <c r="CB4" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="CC4" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="CD4" s="2" t="s">
         <v>14</v>
@@ -4778,16 +4792,16 @@
         <v>14</v>
       </c>
       <c r="CH4" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="CI4" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="CJ4" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="CK4" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="CL4" s="2" t="s">
         <v>14</v>
@@ -4830,7 +4844,7 @@
       </c>
       <c r="CZ4" s="2"/>
     </row>
-    <row r="5" spans="1:104" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:104" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2016</v>
       </c>
@@ -5139,7 +5153,7 @@
       </c>
       <c r="CZ5" s="2"/>
     </row>
-    <row r="6" spans="1:104" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:104" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2017</v>
       </c>
@@ -5448,7 +5462,7 @@
       </c>
       <c r="CZ6" s="2"/>
     </row>
-    <row r="7" spans="1:104" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:104" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2018</v>
       </c>
@@ -5757,7 +5771,7 @@
       </c>
       <c r="CZ7" s="2"/>
     </row>
-    <row r="8" spans="1:104" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:104" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2019</v>
       </c>
@@ -6066,7 +6080,7 @@
       </c>
       <c r="CZ8" s="2"/>
     </row>
-    <row r="9" spans="1:104" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:104" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2020</v>
       </c>
@@ -6375,7 +6389,7 @@
       </c>
       <c r="CZ9" s="2"/>
     </row>
-    <row r="10" spans="1:104" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:104" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2021</v>
       </c>
@@ -6683,7 +6697,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="11" spans="1:104" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:104" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2022</v>
       </c>
@@ -6991,7 +7005,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="12" spans="1:104" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:104" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2023</v>
       </c>
@@ -7299,7 +7313,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="13" spans="1:104" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:104" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2024</v>
       </c>
@@ -7607,7 +7621,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="14" spans="1:104" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:104" x14ac:dyDescent="0.25">
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -7620,7 +7634,7 @@
       <c r="W14" s="2"/>
       <c r="X14" s="2"/>
     </row>
-    <row r="15" spans="1:104" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:104" x14ac:dyDescent="0.25">
       <c r="B15" s="11" t="s">
         <v>14</v>
       </c>
@@ -7640,7 +7654,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:104" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:104" x14ac:dyDescent="0.25">
       <c r="B16" s="5" t="s">
         <v>15</v>
       </c>
@@ -7660,7 +7674,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="2:80" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="2:80" x14ac:dyDescent="0.25">
       <c r="B17" s="6" t="s">
         <v>16</v>
       </c>
@@ -7680,7 +7694,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="2:80" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="2:80" x14ac:dyDescent="0.25">
       <c r="B18" s="7" t="s">
         <v>17</v>
       </c>
@@ -7700,7 +7714,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="2:80" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="2:80" x14ac:dyDescent="0.25">
       <c r="B19" s="9" t="s">
         <v>18</v>
       </c>
@@ -7720,7 +7734,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="2:80" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="2:80" x14ac:dyDescent="0.25">
       <c r="B20" s="8" t="s">
         <v>19</v>
       </c>
@@ -7740,7 +7754,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="2:80" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="2:80" x14ac:dyDescent="0.25">
       <c r="B21" s="10" t="s">
         <v>37</v>
       </c>
@@ -7760,7 +7774,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="2:80" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="2:80" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>20</v>
       </c>
@@ -7782,47 +7796,24 @@
     </row>
   </sheetData>
   <mergeCells count="75">
-    <mergeCell ref="CN2:CO2"/>
-    <mergeCell ref="CP2:CQ2"/>
-    <mergeCell ref="CR2:CS2"/>
-    <mergeCell ref="CT2:CU2"/>
-    <mergeCell ref="CV2:CW2"/>
-    <mergeCell ref="CL2:CM2"/>
-    <mergeCell ref="BP2:BQ2"/>
-    <mergeCell ref="BR2:BS2"/>
-    <mergeCell ref="BT2:BU2"/>
-    <mergeCell ref="BV2:BW2"/>
-    <mergeCell ref="BX2:BY2"/>
-    <mergeCell ref="BZ2:CA2"/>
-    <mergeCell ref="CB2:CC2"/>
-    <mergeCell ref="CD2:CE2"/>
-    <mergeCell ref="CF2:CG2"/>
-    <mergeCell ref="CH2:CI2"/>
-    <mergeCell ref="CJ2:CK2"/>
-    <mergeCell ref="BN2:BO2"/>
-    <mergeCell ref="AR2:AS2"/>
-    <mergeCell ref="AT2:AU2"/>
-    <mergeCell ref="AV2:AW2"/>
-    <mergeCell ref="AX2:AY2"/>
-    <mergeCell ref="AZ2:BA2"/>
-    <mergeCell ref="BB2:BC2"/>
-    <mergeCell ref="BD2:BE2"/>
-    <mergeCell ref="BF2:BG2"/>
-    <mergeCell ref="BH2:BI2"/>
-    <mergeCell ref="BJ2:BK2"/>
-    <mergeCell ref="BL2:BM2"/>
-    <mergeCell ref="AP2:AQ2"/>
-    <mergeCell ref="T2:U2"/>
-    <mergeCell ref="V2:W2"/>
-    <mergeCell ref="X2:Y2"/>
-    <mergeCell ref="Z2:AA2"/>
-    <mergeCell ref="AB2:AC2"/>
-    <mergeCell ref="AD2:AE2"/>
-    <mergeCell ref="AF2:AG2"/>
-    <mergeCell ref="AH2:AI2"/>
-    <mergeCell ref="AJ2:AK2"/>
-    <mergeCell ref="AL2:AM2"/>
-    <mergeCell ref="AN2:AO2"/>
+    <mergeCell ref="V1:Y1"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="J1:M1"/>
+    <mergeCell ref="N1:Q1"/>
+    <mergeCell ref="R1:U1"/>
+    <mergeCell ref="BR1:BU1"/>
+    <mergeCell ref="Z1:AC1"/>
+    <mergeCell ref="AD1:AG1"/>
+    <mergeCell ref="AH1:AK1"/>
+    <mergeCell ref="AL1:AO1"/>
+    <mergeCell ref="AP1:AS1"/>
+    <mergeCell ref="AT1:AW1"/>
+    <mergeCell ref="AX1:BA1"/>
+    <mergeCell ref="BB1:BE1"/>
+    <mergeCell ref="BF1:BI1"/>
+    <mergeCell ref="BJ1:BM1"/>
+    <mergeCell ref="BN1:BQ1"/>
     <mergeCell ref="CT1:CW1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:E2"/>
@@ -7839,24 +7830,47 @@
     <mergeCell ref="CH1:CK1"/>
     <mergeCell ref="CL1:CO1"/>
     <mergeCell ref="CP1:CS1"/>
-    <mergeCell ref="BR1:BU1"/>
-    <mergeCell ref="Z1:AC1"/>
-    <mergeCell ref="AD1:AG1"/>
-    <mergeCell ref="AH1:AK1"/>
-    <mergeCell ref="AL1:AO1"/>
-    <mergeCell ref="AP1:AS1"/>
-    <mergeCell ref="AT1:AW1"/>
-    <mergeCell ref="AX1:BA1"/>
-    <mergeCell ref="BB1:BE1"/>
-    <mergeCell ref="BF1:BI1"/>
-    <mergeCell ref="BJ1:BM1"/>
-    <mergeCell ref="BN1:BQ1"/>
-    <mergeCell ref="V1:Y1"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="J1:M1"/>
-    <mergeCell ref="N1:Q1"/>
-    <mergeCell ref="R1:U1"/>
+    <mergeCell ref="AP2:AQ2"/>
+    <mergeCell ref="T2:U2"/>
+    <mergeCell ref="V2:W2"/>
+    <mergeCell ref="X2:Y2"/>
+    <mergeCell ref="Z2:AA2"/>
+    <mergeCell ref="AB2:AC2"/>
+    <mergeCell ref="AD2:AE2"/>
+    <mergeCell ref="AF2:AG2"/>
+    <mergeCell ref="AH2:AI2"/>
+    <mergeCell ref="AJ2:AK2"/>
+    <mergeCell ref="AL2:AM2"/>
+    <mergeCell ref="AN2:AO2"/>
+    <mergeCell ref="BN2:BO2"/>
+    <mergeCell ref="AR2:AS2"/>
+    <mergeCell ref="AT2:AU2"/>
+    <mergeCell ref="AV2:AW2"/>
+    <mergeCell ref="AX2:AY2"/>
+    <mergeCell ref="AZ2:BA2"/>
+    <mergeCell ref="BB2:BC2"/>
+    <mergeCell ref="BD2:BE2"/>
+    <mergeCell ref="BF2:BG2"/>
+    <mergeCell ref="BH2:BI2"/>
+    <mergeCell ref="BJ2:BK2"/>
+    <mergeCell ref="BL2:BM2"/>
+    <mergeCell ref="CL2:CM2"/>
+    <mergeCell ref="BP2:BQ2"/>
+    <mergeCell ref="BR2:BS2"/>
+    <mergeCell ref="BT2:BU2"/>
+    <mergeCell ref="BV2:BW2"/>
+    <mergeCell ref="BX2:BY2"/>
+    <mergeCell ref="BZ2:CA2"/>
+    <mergeCell ref="CB2:CC2"/>
+    <mergeCell ref="CD2:CE2"/>
+    <mergeCell ref="CF2:CG2"/>
+    <mergeCell ref="CH2:CI2"/>
+    <mergeCell ref="CJ2:CK2"/>
+    <mergeCell ref="CN2:CO2"/>
+    <mergeCell ref="CP2:CQ2"/>
+    <mergeCell ref="CR2:CS2"/>
+    <mergeCell ref="CT2:CU2"/>
+    <mergeCell ref="CV2:CW2"/>
   </mergeCells>
   <conditionalFormatting sqref="B4:CW13">
     <cfRule type="cellIs" dxfId="12" priority="1" operator="equal">
@@ -7892,14 +7906,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{221F9016-2A40-4C0A-A371-63EB68CE326F}">
   <dimension ref="A1:K26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="10.26171875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.68359375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.1015625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -7934,7 +7948,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -7972,7 +7986,7 @@
       </c>
       <c r="K2" s="2"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <f>A2+1</f>
         <v>2</v>
@@ -8011,7 +8025,7 @@
       </c>
       <c r="K3" s="2"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" ref="A4:A26" si="4">A3+1</f>
         <v>3</v>
@@ -8052,7 +8066,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="4"/>
         <v>4</v>
@@ -8091,7 +8105,7 @@
       </c>
       <c r="K5" s="2"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="4"/>
         <v>5</v>
@@ -8130,7 +8144,7 @@
       </c>
       <c r="K6" s="2"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7">
         <f t="shared" si="4"/>
         <v>6</v>
@@ -8169,7 +8183,7 @@
       </c>
       <c r="K7" s="2"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8">
         <f t="shared" si="4"/>
         <v>7</v>
@@ -8208,7 +8222,7 @@
       </c>
       <c r="K8" s="2"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9">
         <f t="shared" si="4"/>
         <v>8</v>
@@ -8247,7 +8261,7 @@
       </c>
       <c r="K9" s="2"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10">
         <f t="shared" si="4"/>
         <v>9</v>
@@ -8286,7 +8300,7 @@
       </c>
       <c r="K10" s="2"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11">
         <f t="shared" si="4"/>
         <v>10</v>
@@ -8325,7 +8339,7 @@
       </c>
       <c r="K11" s="2"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12">
         <f t="shared" si="4"/>
         <v>11</v>
@@ -8364,7 +8378,7 @@
       </c>
       <c r="K12" s="2"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13">
         <f t="shared" si="4"/>
         <v>12</v>
@@ -8404,7 +8418,7 @@
       </c>
       <c r="K13" s="2"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14">
         <f t="shared" si="4"/>
         <v>13</v>
@@ -8443,7 +8457,7 @@
       </c>
       <c r="K14" s="2"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15">
         <f t="shared" si="4"/>
         <v>14</v>
@@ -8485,7 +8499,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16">
         <f t="shared" si="4"/>
         <v>15</v>
@@ -8524,7 +8538,7 @@
       </c>
       <c r="K16" s="2"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17">
         <f t="shared" si="4"/>
         <v>16</v>
@@ -8563,7 +8577,7 @@
       </c>
       <c r="K17" s="2"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18">
         <f t="shared" si="4"/>
         <v>17</v>
@@ -8602,7 +8616,7 @@
       </c>
       <c r="K18" s="2"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19">
         <f t="shared" si="4"/>
         <v>18</v>
@@ -8641,7 +8655,7 @@
       </c>
       <c r="K19" s="2"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20">
         <f t="shared" si="4"/>
         <v>19</v>
@@ -8680,7 +8694,7 @@
       </c>
       <c r="K20" s="2"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21">
         <f t="shared" si="4"/>
         <v>20</v>
@@ -8719,7 +8733,7 @@
       </c>
       <c r="K21" s="2"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22">
         <f t="shared" si="4"/>
         <v>21</v>
@@ -8761,7 +8775,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23">
         <f t="shared" si="4"/>
         <v>22</v>
@@ -8800,7 +8814,7 @@
       </c>
       <c r="K23" s="2"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24">
         <f t="shared" si="4"/>
         <v>23</v>
@@ -8839,7 +8853,7 @@
       </c>
       <c r="K24" s="2"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25">
         <f t="shared" si="4"/>
         <v>24</v>
@@ -8879,7 +8893,7 @@
       </c>
       <c r="K25" s="2"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26">
         <f t="shared" si="4"/>
         <v>25</v>
@@ -8980,9 +8994,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3A3E9AF-60E4-42C2-9582-F318C9A6FCBA}">
   <dimension ref="A1:J26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -9014,7 +9028,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -9051,7 +9065,7 @@
         <v>0.10090837190364987</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
         <f>A2+1</f>
         <v>2</v>
@@ -9089,7 +9103,7 @@
         <v>0.14716935215907975</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" ref="A4:A26" si="4">A3+1</f>
         <v>3</v>
@@ -9127,7 +9141,7 @@
         <v>0.14737526851024199</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="4"/>
         <v>4</v>
@@ -9165,7 +9179,7 @@
         <v>9.4169291320157805E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="4"/>
         <v>5</v>
@@ -9203,7 +9217,7 @@
         <v>0.14031327364879095</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7">
         <f t="shared" si="4"/>
         <v>6</v>
@@ -9241,7 +9255,7 @@
         <v>0.20000561590048624</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8">
         <f t="shared" si="4"/>
         <v>7</v>
@@ -9279,7 +9293,7 @@
         <v>0.10944922055981168</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9">
         <f t="shared" si="4"/>
         <v>8</v>
@@ -9317,7 +9331,7 @@
         <v>0.11353946808062561</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10">
         <f t="shared" si="4"/>
         <v>9</v>
@@ -9355,7 +9369,7 @@
         <v>7.5454302949751736E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11">
         <f t="shared" si="4"/>
         <v>10</v>
@@ -9393,7 +9407,7 @@
         <v>0.11180789876403389</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12">
         <f t="shared" si="4"/>
         <v>11</v>
@@ -9423,7 +9437,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13">
         <f t="shared" si="4"/>
         <v>12</v>
@@ -9453,7 +9467,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14">
         <f t="shared" si="4"/>
         <v>13</v>
@@ -9483,7 +9497,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15">
         <f t="shared" si="4"/>
         <v>14</v>
@@ -9513,7 +9527,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16">
         <f t="shared" si="4"/>
         <v>15</v>
@@ -9543,7 +9557,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17">
         <f t="shared" si="4"/>
         <v>16</v>
@@ -9573,7 +9587,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18">
         <f t="shared" si="4"/>
         <v>17</v>
@@ -9603,7 +9617,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19">
         <f t="shared" si="4"/>
         <v>18</v>
@@ -9633,7 +9647,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20">
         <f t="shared" si="4"/>
         <v>19</v>
@@ -9663,7 +9677,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21">
         <f t="shared" si="4"/>
         <v>20</v>
@@ -9693,7 +9707,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22">
         <f t="shared" si="4"/>
         <v>21</v>
@@ -9723,7 +9737,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23">
         <f t="shared" si="4"/>
         <v>22</v>
@@ -9753,7 +9767,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24">
         <f t="shared" si="4"/>
         <v>23</v>
@@ -9783,7 +9797,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25">
         <f t="shared" si="4"/>
         <v>24</v>
@@ -9813,7 +9827,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26">
         <f t="shared" si="4"/>
         <v>25</v>
@@ -9904,13 +9918,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.41796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -9942,7 +9956,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -9979,7 +9993,7 @@
         <v>0.12656050665208676</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
         <f>A2+1</f>
         <v>2</v>
@@ -10017,7 +10031,7 @@
         <v>0.15704733916529981</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" ref="A4:A26" si="4">A3+1</f>
         <v>3</v>
@@ -10055,7 +10069,7 @@
         <v>9.0082239839620923E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="4"/>
         <v>4</v>
@@ -10093,7 +10107,7 @@
         <v>8.8470475669764903E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="4"/>
         <v>5</v>
@@ -10131,7 +10145,7 @@
         <v>0.25705645161290325</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7">
         <f t="shared" si="4"/>
         <v>6</v>
@@ -10169,7 +10183,7 @@
         <v>0.11689561691270275</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8">
         <f t="shared" si="4"/>
         <v>7</v>
@@ -10207,7 +10221,7 @@
         <v>0.12984668306907235</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9">
         <f t="shared" si="4"/>
         <v>8</v>
@@ -10245,7 +10259,7 @@
         <v>0.11064219974485147</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10">
         <f t="shared" si="4"/>
         <v>9</v>
@@ -10283,7 +10297,7 @@
         <v>9.2764716602879535E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11">
         <f t="shared" si="4"/>
         <v>10</v>
@@ -10321,7 +10335,7 @@
         <v>0.10031665755421906</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12">
         <f t="shared" si="4"/>
         <v>11</v>
@@ -10359,7 +10373,7 @@
         <v>9.8989657371970116E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13">
         <f t="shared" si="4"/>
         <v>12</v>
@@ -10397,7 +10411,7 @@
         <v>6.7175824676508109E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14">
         <f t="shared" si="4"/>
         <v>13</v>
@@ -10435,7 +10449,7 @@
         <v>6.6019682886823403E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15">
         <f t="shared" si="4"/>
         <v>14</v>
@@ -10473,7 +10487,7 @@
         <v>0.11193502824858757</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16">
         <f t="shared" si="4"/>
         <v>15</v>
@@ -10503,7 +10517,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17">
         <f t="shared" si="4"/>
         <v>16</v>
@@ -10533,7 +10547,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18">
         <f t="shared" si="4"/>
         <v>17</v>
@@ -10563,7 +10577,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19">
         <f t="shared" si="4"/>
         <v>18</v>
@@ -10593,7 +10607,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20">
         <f t="shared" si="4"/>
         <v>19</v>
@@ -10623,7 +10637,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21">
         <f t="shared" si="4"/>
         <v>20</v>
@@ -10653,7 +10667,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22">
         <f t="shared" si="4"/>
         <v>21</v>
@@ -10683,7 +10697,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23">
         <f t="shared" si="4"/>
         <v>22</v>
@@ -10713,7 +10727,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24">
         <f t="shared" si="4"/>
         <v>23</v>
@@ -10743,7 +10757,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25">
         <f t="shared" si="4"/>
         <v>24</v>
@@ -10773,7 +10787,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26">
         <f t="shared" si="4"/>
         <v>25</v>
@@ -10863,13 +10877,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="7" max="8" width="8.83984375" style="1"/>
-    <col min="10" max="10" width="11.15625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="8.85546875" style="1"/>
+    <col min="10" max="10" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -10901,7 +10915,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -10938,7 +10952,7 @@
         <v>0.16424822307271733</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
         <f>A2+1</f>
         <v>2</v>
@@ -10976,7 +10990,7 @@
         <v>0.20143247676325862</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" ref="A4:A26" si="2">A3+1</f>
         <v>3</v>
@@ -11014,7 +11028,7 @@
         <v>0.15932203389830507</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="2"/>
         <v>4</v>
@@ -11052,7 +11066,7 @@
         <v>0.12741388737014761</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="2"/>
         <v>5</v>
@@ -11090,7 +11104,7 @@
         <v>0.12896118097320941</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7">
         <f t="shared" si="2"/>
         <v>6</v>
@@ -11128,7 +11142,7 @@
         <v>0.1137834882449426</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8">
         <f t="shared" si="2"/>
         <v>7</v>
@@ -11166,7 +11180,7 @@
         <v>8.9409513395297971E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9">
         <f t="shared" si="2"/>
         <v>8</v>
@@ -11204,7 +11218,7 @@
         <v>7.9158009841443416E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10">
         <f t="shared" si="2"/>
         <v>9</v>
@@ -11242,7 +11256,7 @@
         <v>9.1623838162930557E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11">
         <f t="shared" si="2"/>
         <v>10</v>
@@ -11280,7 +11294,7 @@
         <v>5.7851284855112081E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12">
         <f t="shared" si="2"/>
         <v>11</v>
@@ -11318,7 +11332,7 @@
         <v>8.3105522143247679E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13">
         <f t="shared" si="2"/>
         <v>12</v>
@@ -11356,7 +11370,7 @@
         <v>6.6790595954073259E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14">
         <f t="shared" si="2"/>
         <v>13</v>
@@ -11394,7 +11408,7 @@
         <v>4.8693275013668672E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15">
         <f t="shared" si="2"/>
         <v>14</v>
@@ -11432,7 +11446,7 @@
         <v>6.8316019682886822E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16">
         <f t="shared" si="2"/>
         <v>15</v>
@@ -11470,7 +11484,7 @@
         <v>4.6074357572443957E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17">
         <f t="shared" si="2"/>
         <v>16</v>
@@ -11508,7 +11522,7 @@
         <v>6.3860032804811367E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18">
         <f t="shared" si="2"/>
         <v>17</v>
@@ -11546,7 +11560,7 @@
         <v>6.762165117550574E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19">
         <f t="shared" si="2"/>
         <v>18</v>
@@ -11584,7 +11598,7 @@
         <v>8.3838162930563148E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20">
         <f t="shared" si="2"/>
         <v>19</v>
@@ -11622,7 +11636,7 @@
         <v>9.9382176052487697E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21">
         <f t="shared" si="2"/>
         <v>20</v>
@@ -11660,7 +11674,7 @@
         <v>8.2400218698742478E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22">
         <f t="shared" si="2"/>
         <v>21</v>
@@ -11698,7 +11712,7 @@
         <v>3.9404045926735923E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23">
         <f t="shared" si="2"/>
         <v>22</v>
@@ -11736,7 +11750,7 @@
         <v>3.9704756697648988E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24">
         <f t="shared" si="2"/>
         <v>23</v>
@@ -11774,7 +11788,7 @@
         <v>3.693821760524877E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25">
         <f t="shared" si="2"/>
         <v>24</v>
@@ -11812,7 +11826,7 @@
         <v>4.5095680699835973E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26">
         <f t="shared" si="2"/>
         <v>25</v>
@@ -11914,13 +11928,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:J26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="7" max="8" width="9.15625" style="1"/>
-    <col min="10" max="10" width="11.15625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="9.140625" style="1"/>
+    <col min="10" max="10" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -11952,7 +11966,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -11989,7 +12003,7 @@
         <v>0.19788460512035869</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
         <f>A2+1</f>
         <v>2</v>
@@ -12027,7 +12041,7 @@
         <v>7.4092194922340635E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" ref="A4:A26" si="2">A3+1</f>
         <v>3</v>
@@ -12065,7 +12079,7 @@
         <v>4.3179675129432278E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="2"/>
         <v>4</v>
@@ -12103,7 +12117,7 @@
         <v>9.5628658352162541E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="2"/>
         <v>5</v>
@@ -12141,7 +12155,7 @@
         <v>4.1169249381749602E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7">
         <f t="shared" si="2"/>
         <v>6</v>
@@ -12179,7 +12193,7 @@
         <v>7.0453858060383942E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8">
         <f t="shared" si="2"/>
         <v>7</v>
@@ -12217,7 +12231,7 @@
         <v>4.9406657533759141E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9">
         <f t="shared" si="2"/>
         <v>8</v>
@@ -12255,7 +12269,7 @@
         <v>5.1772910847403347E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10">
         <f t="shared" si="2"/>
         <v>9</v>
@@ -12293,7 +12307,7 @@
         <v>4.995819026099952E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11">
         <f t="shared" si="2"/>
         <v>10</v>
@@ -12331,7 +12345,7 @@
         <v>7.870905759069155E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12">
         <f t="shared" si="2"/>
         <v>11</v>
@@ -12369,7 +12383,7 @@
         <v>4.2129983809845749E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13">
         <f t="shared" si="2"/>
         <v>12</v>
@@ -12407,7 +12421,7 @@
         <v>2.9480313839913178E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14">
         <f t="shared" si="2"/>
         <v>13</v>
@@ -12445,7 +12459,7 @@
         <v>2.3173270233244968E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15">
         <f t="shared" si="2"/>
         <v>14</v>
@@ -12483,7 +12497,7 @@
         <v>2.4641058942836302E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16">
         <f t="shared" si="2"/>
         <v>15</v>
@@ -12515,7 +12529,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17">
         <f t="shared" si="2"/>
         <v>16</v>
@@ -12553,7 +12567,7 @@
         <v>3.2451474015691997E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18">
         <f t="shared" si="2"/>
         <v>17</v>
@@ -12591,7 +12605,7 @@
         <v>2.5379401142206486E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19">
         <f t="shared" si="2"/>
         <v>18</v>
@@ -12623,7 +12637,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20">
         <f t="shared" si="2"/>
         <v>19</v>
@@ -12661,7 +12675,7 @@
         <v>2.0335545394701726E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21">
         <f t="shared" si="2"/>
         <v>20</v>
@@ -12693,7 +12707,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22">
         <f t="shared" si="2"/>
         <v>21</v>
@@ -12725,7 +12739,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23">
         <f t="shared" si="2"/>
         <v>22</v>
@@ -12760,7 +12774,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24">
         <f t="shared" si="2"/>
         <v>23</v>
@@ -12792,7 +12806,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25">
         <f t="shared" si="2"/>
         <v>24</v>
@@ -12824,7 +12838,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26">
         <f t="shared" si="2"/>
         <v>25</v>
@@ -12920,13 +12934,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:J26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="7" max="8" width="9.15625" style="1"/>
-    <col min="10" max="10" width="11.15625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="9.140625" style="1"/>
+    <col min="10" max="10" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -12958,7 +12972,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -12995,7 +13009,7 @@
         <v>7.9995509654243374E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
         <f>A2+1</f>
         <v>2</v>
@@ -13033,7 +13047,7 @@
         <v>0.24185002245172879</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" ref="A4:A26" si="2">A3+1</f>
         <v>3</v>
@@ -13071,7 +13085,7 @@
         <v>7.9872025145936235E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="2"/>
         <v>4</v>
@@ -13109,7 +13123,7 @@
         <v>6.8702290076335881E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="2"/>
         <v>5</v>
@@ -13147,7 +13161,7 @@
         <v>8.1960035922766059E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7">
         <f t="shared" si="2"/>
         <v>6</v>
@@ -13185,7 +13199,7 @@
         <v>4.5229007633587788E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8">
         <f t="shared" si="2"/>
         <v>7</v>
@@ -13223,7 +13237,7 @@
         <v>3.6517736865738663E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9">
         <f t="shared" si="2"/>
         <v>8</v>
@@ -13261,7 +13275,7 @@
         <v>5.0437808711270765E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10">
         <f t="shared" si="2"/>
         <v>9</v>
@@ -13299,7 +13313,7 @@
         <v>6.5514144589133363E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11">
         <f t="shared" si="2"/>
         <v>10</v>
@@ -13337,7 +13351,7 @@
         <v>5.004490345756623E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12">
         <f t="shared" si="2"/>
         <v>11</v>
@@ -13375,7 +13389,7 @@
         <v>5.3682083520431072E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13">
         <f t="shared" si="2"/>
         <v>12</v>
@@ -13413,7 +13427,7 @@
         <v>3.3464301751234847E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14">
         <f t="shared" si="2"/>
         <v>13</v>
@@ -13451,7 +13465,7 @@
         <v>5.9744050291872478E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15">
         <f t="shared" si="2"/>
         <v>14</v>
@@ -13489,7 +13503,7 @@
         <v>5.4086214638527169E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16">
         <f t="shared" si="2"/>
         <v>15</v>
@@ -13527,7 +13541,7 @@
         <v>2.2968118545127973E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17">
         <f t="shared" si="2"/>
         <v>16</v>
@@ -13565,7 +13579,7 @@
         <v>3.7853614728334081E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18">
         <f t="shared" si="2"/>
         <v>17</v>
@@ -13603,7 +13617,7 @@
         <v>3.022002694207454E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19">
         <f t="shared" si="2"/>
         <v>18</v>
@@ -13641,7 +13655,7 @@
         <v>4.64863044454423E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20">
         <f t="shared" si="2"/>
         <v>19</v>
@@ -13679,7 +13693,7 @@
         <v>3.8381230354737318E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21">
         <f t="shared" si="2"/>
         <v>20</v>
@@ -13717,7 +13731,7 @@
         <v>3.082622361921868E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22">
         <f t="shared" si="2"/>
         <v>21</v>
@@ -13755,7 +13769,7 @@
         <v>2.9726088908845982E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23">
         <f t="shared" si="2"/>
         <v>22</v>
@@ -13793,7 +13807,7 @@
         <v>3.0377189043556355E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24">
         <f t="shared" si="2"/>
         <v>23</v>
@@ -13831,7 +13845,7 @@
         <v>3.2611136057476425E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25">
         <f t="shared" si="2"/>
         <v>24</v>
@@ -13869,7 +13883,7 @@
         <v>3.2476425684777731E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26">
         <f t="shared" si="2"/>
         <v>25</v>
@@ -13967,13 +13981,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:J26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="7" max="8" width="9.15625" style="1"/>
-    <col min="10" max="10" width="11.15625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="9.140625" style="1"/>
+    <col min="10" max="10" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -14005,7 +14019,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -14042,7 +14056,7 @@
         <v>0.10645998481665225</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
         <f>A2+1</f>
         <v>2</v>
@@ -14080,7 +14094,7 @@
         <v>0.11230380819547678</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" ref="A4:A26" si="4">A3+1</f>
         <v>3</v>
@@ -14118,7 +14132,7 @@
         <v>0.15672392789675324</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="4"/>
         <v>4</v>
@@ -14156,7 +14170,7 @@
         <v>0.11124450486396779</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="4"/>
         <v>5</v>
@@ -14194,7 +14208,7 @@
         <v>0.1321657456612701</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7">
         <f t="shared" si="4"/>
         <v>6</v>
@@ -14232,7 +14246,7 @@
         <v>0.11818294168535159</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8">
         <f t="shared" si="4"/>
         <v>7</v>
@@ -14270,7 +14284,7 @@
         <v>0.13804487915114494</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9">
         <f t="shared" si="4"/>
         <v>8</v>
@@ -14308,7 +14322,7 @@
         <v>0.11504034180187497</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10">
         <f t="shared" si="4"/>
         <v>9</v>
@@ -14346,7 +14360,7 @@
         <v>7.6658251090199678E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11">
         <f t="shared" si="4"/>
         <v>10</v>
@@ -14384,7 +14398,7 @@
         <v>6.3046203280309313E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12">
         <f t="shared" si="4"/>
         <v>11</v>
@@ -14422,7 +14436,7 @@
         <v>6.5341360498578763E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13">
         <f t="shared" si="4"/>
         <v>12</v>
@@ -14460,7 +14474,7 @@
         <v>7.9747885807100863E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14">
         <f t="shared" si="4"/>
         <v>13</v>
@@ -14498,7 +14512,7 @@
         <v>7.1061598488727243E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15">
         <f t="shared" si="4"/>
         <v>14</v>
@@ -14536,7 +14550,7 @@
         <v>8.2096008191945763E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16">
         <f t="shared" si="4"/>
         <v>15</v>
@@ -14574,7 +14588,7 @@
         <v>5.2347239632068644E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17">
         <f t="shared" si="4"/>
         <v>16</v>
@@ -14612,7 +14626,7 @@
         <v>7.1767800709733237E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18">
         <f t="shared" si="4"/>
         <v>17</v>
@@ -14650,7 +14664,7 @@
         <v>5.0581734079553679E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19">
         <f t="shared" si="4"/>
         <v>18</v>
@@ -14688,7 +14702,7 @@
         <v>4.4702600589678856E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20">
         <f t="shared" si="4"/>
         <v>19</v>
@@ -14726,7 +14740,7 @@
         <v>4.7915820695256087E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21">
         <f t="shared" si="4"/>
         <v>20</v>
@@ -14764,7 +14778,7 @@
         <v>4.7968785861831537E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22">
         <f t="shared" si="4"/>
         <v>21</v>
@@ -14802,7 +14816,7 @@
         <v>5.1376211578185414E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23">
         <f t="shared" si="4"/>
         <v>22</v>
@@ -14840,7 +14854,7 @@
         <v>5.8967885453999752E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24">
         <f t="shared" si="4"/>
         <v>23</v>
@@ -14878,7 +14892,7 @@
         <v>3.1867375222895074E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25">
         <f t="shared" si="4"/>
         <v>24</v>
@@ -14916,7 +14930,7 @@
         <v>3.7110926713864519E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26">
         <f t="shared" si="4"/>
         <v>25</v>

</xml_diff>